<commit_message>
Yearly skills intervention scenario
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="7">
   <si>
     <t>Country</t>
   </si>
@@ -30,6 +30,9 @@
   </si>
   <si>
     <t>2011</t>
+  </si>
+  <si>
+    <t>2018</t>
   </si>
 </sst>
 </file>
@@ -90,7 +93,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated init pop files and SkillsInterventionFlag
</commit_message>
<xml_diff>
--- a/input/DatabaseCountryYear.xlsx
+++ b/input/DatabaseCountryYear.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="8">
   <si>
     <t>Country</t>
   </si>
@@ -30,6 +30,12 @@
   </si>
   <si>
     <t>2011</t>
+  </si>
+  <si>
+    <t>2018</t>
+  </si>
+  <si>
+    <t>2023</t>
   </si>
 </sst>
 </file>
@@ -90,7 +96,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>